<commit_message>
update jobs and conference
</commit_message>
<xml_diff>
--- a/about/committees.xlsx
+++ b/about/committees.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emma/docs/apls-org/about/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EDFB39B9-4891-1349-AD47-13A7F190A139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB5BC034-4CA0-0248-B5FC-D52152B613C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34560" yWindow="1640" windowWidth="27640" windowHeight="16940" xr2:uid="{7EC594C2-72CE-094E-8270-448939084E54}"/>
+    <workbookView xWindow="2980" yWindow="680" windowWidth="26540" windowHeight="18960" xr2:uid="{7EC594C2-72CE-094E-8270-448939084E54}"/>
   </bookViews>
   <sheets>
     <sheet name="committees" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="234">
   <si>
     <t>key</t>
   </si>
@@ -535,30 +535,6 @@
     <t>SciencePaper</t>
   </si>
   <si>
-    <t>Scientific Paper Review Committee</t>
-  </si>
-  <si>
-    <t>The committee oversees the process by which scientific review papers (or white papers) are prepared, reviewed and approved. Only those topics that are approved by the Executive Committee of AP-LS will be considered for a white paper. The committee chair is responsible for appointing the lead author, working with the lead author, and approving additional members of the writing group. The committee chair will ensure that the process involves extensive opportunities for wide input from AP-LS members, which will normally include postings of a draft for AP-LS member comments, presentation of the paper at an AP-LS annual conference meeting, and targeted reviews by other experts solicited by the committee chair as appropriate, including the editor of Law and Human Behavior. The manuscript will be submitted to Law and Human Behavior for publication and requires approval of the Executive Committee of AP-LS before it becomes an official scientific review paper of AP-LS.</t>
-  </si>
-  <si>
-    <t>The Committee oversees the process by which scientific review papers (or ‚Äúwhite papers‚Äù) are prepared, reviewed, and approved. Only those topics that are approved by the Executive Committee of AP-LS will be considered for a white paper. The Committee Chair is responsible for appointing the lead author, working with the lead author, and approving additional members of the writing group. The Committee Chair will ensure that the process involves extensive opportunities for wide input from AP-LS members, which will normally include postings of a draft for AP-LS member comments, presentation of the paper at an AP-LS annual conference meeting, and targeted reviews by other experts solicited by the Committee Chair as appropriate, including the Editor of Law and Human Behavior. The manuscript will be submitted to Law and Human Behavior for publication and requires approval of the Executive Committee of AP-LS before it becomes an official scientific review paper of AP-LS.</t>
-  </si>
-  <si>
-    <t>The Scientific Review Paper Committee supports the following aspects of the AP-LS Mission: A unifying force for psychology-law science and practice; the major catalyst for the stimulation and growth and dissemination of psychology-law science and practice; the primary resource for all psychology-law scholars and practitioners and for members of other disciplines with interest in psychology-law science and practice; the leading advocate for psychology-law knowledge and practice informing practitioners, policy makers and the public to use psychology-law knowledge in the pursuit of justice for all citizens; a principle leader and global partner promoting psychology-law knowledge and methods to improve justice in diverse, multicultural and international contexts; and an effective champion of the application of psychology-law to promote human rights, dignity and justice. The Scientific Review Paper Committee also supports the AP-LS Core Values of: continual pursuit of excellence; knowledge and application based on methods of science; outstanding service to its members and to society; and social justice, diversity and inclusion; and ethical action in all that we do.</t>
-  </si>
-  <si>
-    <t>There are no scheduled meetings.</t>
-  </si>
-  <si>
-    <t>There is a standing Committee Chair, but the extended committee is ad hoc for any given paper and is composed of those who write the paper. The Chair and committee members are appointed by the AP-LS President.</t>
-  </si>
-  <si>
-    <t>The Committee provides a semi-annual written report to the Executive Committee as requested by the AP-LS President. The Chair attends the Executive Committee meeting to discuss the report as needed.</t>
-  </si>
-  <si>
-    <t>There have been only two scientific review papers in AP-LS history, one on eyewitness identification and one on confessions. The general attitude of the Executive Committee and the current and previous Chair of the Scientific Review Paper Committee can be described as very conservative. A topic must reach a rather high point of scientific clarity and consensus among AP-LS members to justify consideration.</t>
-  </si>
-  <si>
     <t>Lindsay Malloy</t>
   </si>
   <si>
@@ -725,13 +701,114 @@
   </si>
   <si>
     <t>The PDW Committee is responsible for promoting the success and professional development of female scientists and practitioners in the field of legal/forensic psychology. By identifying and addressing potential obstacles to career advancement, the committee hopes to promote better representation of women at all levels of academic and professional rank and greater recognition of womens achievement in AP-LS and AAFP. To meet this objective, the PDW Committee provides support, mentorship, and training to AP-LS members through meetings at the annual AP-LS conference and via a blog overseen by members of the committee. On occasion, the PDW Committee may also survey the membership to assess needs of the membership and to monitor the challenges/successes of both men and women in the field.</t>
+  </si>
+  <si>
+    <t>Scientific Review Paper Committee</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The committee oversees the process by which scientific review papers are prepared, reviewed, and approved. Only those topics that are approved by the Executive Committee of the AP-LS will be considered for a scientific review paper. The committee chair is responsible for appointing the lead author, working with the lead author, and approving additional members of the writing group. The committee chair will ensure that the process involves extensive opportunities for wide input from AP-LS members, which will normally include postings of a draft for the AP-LS member comments, presentations of the paper at an AP-LS and an APA annual conference meeting, and targeted reviews by other experts solicited by the committee chair as appropriate, including the editor of </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Law and Human Behavior</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">. The manuscript will be submitted to </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Law and Human Behavior</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> for publication and requires approval of the Executive Committee of AP-LS before it becomes an official scientific review paper of the AP-LS.</t>
+    </r>
+  </si>
+  <si>
+    <t>The Scientific Review Paper Committee supports the following aspects of the AP-LS mission: A unifying force for psychology-law science and practice; the major catalyst for the stimulation and growth and dissemination of psychology-law science and practice; the primary resource for all psychology-law scholars and practitioners and for members of other disciplines with interest in psychology-law science and practice; the leading advocate for psychology-law knowledge and practice informing practitioners, policymakers, and the public to use psychology-law knowledge in the pursuit of justice for all citizens; a principle leader and global partner promoting psychology-law knowledge and methods to improve justice in diverse, multicultural and international contexts; and an effective champion of the application of psychology-law to promote human rights, dignity, and justice. The Scientific Review Paper Committee also supports the AP-LS core values of: continual pursuit of excellence; knowledge and application based on methods of science; outstanding service to its members and to society; social justice, diversity and inclusion; and ethical action in all that we do. Scientific Review Paper topics must reach a high point of scientific clarity and consensus among the AP-LS members to justify consideration.</t>
+  </si>
+  <si>
+    <t>The SRP chair and committee members meet on an as-needed basis.</t>
+  </si>
+  <si>
+    <r>
+      <t>The Committee consists of a Chair and additional AP-LS members as determined by the committee needs. The Chair and Members are appointed by the AP-LS President and typically serve 3-year terms each. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Committee members should be relatively senior in the field. T</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">o the extent possible, members of the committee should ideally represent different areas of research and/or practice. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Typically, the Chair of the SRP committee is first designated by their fellow SRP committee members and then officially appointed by the AP-LS President. </t>
+    </r>
+  </si>
+  <si>
+    <t>The Committee provides a semi-annual written report to the Executive Committee as requested by the AP-LS President. The Chair attends the Executive Committee meetings to discuss the report as needed.   </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">In 1995, the AP-LS Executive Committee approved an initiative to ‘‘write Scientific Review Papers summarizing the psychological research in specific policy areas’’ (Wiener, 1998). The key goals are: 1) to objectively summarize the research literature in areas where there is a high degree of scientific clarity and consensus; and 2) to serve as a science translation document, providing guidelines and recommendations useful to police, lawyers, judges, legislators, and the public. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF222222"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>The Scientific Review Paper (SRP) Committee also supports the AP-LS core values of: continual pursuit of excellence; knowledge and application based on methods of science; outstanding service to its members and to society; social justice, diversity and inclusion; and ethical action in all that we do. Learn more about the SRC process at this link: https://h7.cl/1gFs2</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -865,6 +942,37 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF222222"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1208,8 +1316,18 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1698,7 +1816,7 @@
         <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="E4" t="s">
         <v>33</v>
@@ -1727,7 +1845,7 @@
         <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="D5" t="s">
         <v>41</v>
@@ -1823,10 +1941,10 @@
         <v>69</v>
       </c>
       <c r="D8" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="E8" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="F8" t="s">
         <v>70</v>
@@ -1890,7 +2008,7 @@
         <v>87</v>
       </c>
       <c r="E10" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="F10" t="s">
         <v>88</v>
@@ -2064,10 +2182,10 @@
         <v>139</v>
       </c>
       <c r="C16" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="D16" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="E16" t="s">
         <v>140</v>
@@ -2180,170 +2298,167 @@
         <v>170</v>
       </c>
       <c r="B20" t="s">
+        <v>227</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="J20" t="s">
         <v>171</v>
       </c>
-      <c r="C20" t="s">
+      <c r="K20" t="s">
         <v>172</v>
-      </c>
-      <c r="D20" t="s">
-        <v>173</v>
-      </c>
-      <c r="E20" t="s">
-        <v>174</v>
-      </c>
-      <c r="F20" t="s">
-        <v>175</v>
-      </c>
-      <c r="G20" t="s">
-        <v>176</v>
-      </c>
-      <c r="H20" t="s">
-        <v>177</v>
-      </c>
-      <c r="I20" t="s">
-        <v>178</v>
-      </c>
-      <c r="J20" t="s">
-        <v>179</v>
-      </c>
-      <c r="K20" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>173</v>
+      </c>
+      <c r="B21" t="s">
+        <v>174</v>
+      </c>
+      <c r="C21" t="s">
+        <v>175</v>
+      </c>
+      <c r="E21" t="s">
+        <v>176</v>
+      </c>
+      <c r="F21" t="s">
+        <v>177</v>
+      </c>
+      <c r="G21" t="s">
+        <v>178</v>
+      </c>
+      <c r="H21" t="s">
+        <v>179</v>
+      </c>
+      <c r="J21" t="s">
+        <v>180</v>
+      </c>
+      <c r="K21" t="s">
         <v>181</v>
-      </c>
-      <c r="B21" t="s">
-        <v>182</v>
-      </c>
-      <c r="C21" t="s">
-        <v>183</v>
-      </c>
-      <c r="E21" t="s">
-        <v>184</v>
-      </c>
-      <c r="F21" t="s">
-        <v>185</v>
-      </c>
-      <c r="G21" t="s">
-        <v>186</v>
-      </c>
-      <c r="H21" t="s">
-        <v>187</v>
-      </c>
-      <c r="J21" t="s">
-        <v>188</v>
-      </c>
-      <c r="K21" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="B22" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="C22" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="J22" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="K22" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="B23" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="C23" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="D23" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="E23" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="F23" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="G23" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="H23" t="s">
         <v>55</v>
       </c>
       <c r="J23" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="K23" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="B24" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="C24" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D24" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E24" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="F24" t="s">
         <v>116</v>
       </c>
       <c r="G24" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="H24" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="J24" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="K24" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="B25" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C25" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="D25" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="E25" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="F25" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="G25" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="H25" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="J25" t="s">
         <v>168</v>
@@ -2354,25 +2469,25 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="B26" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="C26" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="E26" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="F26" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="G26" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="H26" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update awards, jobs, conference archive and SRP
</commit_message>
<xml_diff>
--- a/about/committees.xlsx
+++ b/about/committees.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emma/docs/apls-org/about/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB5BC034-4CA0-0248-B5FC-D52152B613C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05822146-6248-AB4A-A3CF-6D9735D39DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2980" yWindow="680" windowWidth="26540" windowHeight="18960" xr2:uid="{7EC594C2-72CE-094E-8270-448939084E54}"/>
+    <workbookView xWindow="3300" yWindow="660" windowWidth="26240" windowHeight="18980" xr2:uid="{7EC594C2-72CE-094E-8270-448939084E54}"/>
   </bookViews>
   <sheets>
     <sheet name="committees" sheetId="1" r:id="rId1"/>
@@ -533,12 +533,6 @@
   </si>
   <si>
     <t>SciencePaper</t>
-  </si>
-  <si>
-    <t>Lindsay Malloy</t>
-  </si>
-  <si>
-    <t>Lindsay.malloy@ontariotechu.ca</t>
   </si>
   <si>
     <t>SocialMedia</t>
@@ -790,6 +784,12 @@
     <t>The Committee provides a semi-annual written report to the Executive Committee as requested by the AP-LS President. The Chair attends the Executive Committee meetings to discuss the report as needed.   </t>
   </si>
   <si>
+    <t xml:space="preserve">r_fitzgerald@sfu.ca </t>
+  </si>
+  <si>
+    <t>Ryan Fitzgerald</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">In 1995, the AP-LS Executive Committee approved an initiative to ‘‘write Scientific Review Papers summarizing the psychological research in specific policy areas’’ (Wiener, 1998). The key goals are: 1) to objectively summarize the research literature in areas where there is a high degree of scientific clarity and consensus; and 2) to serve as a science translation document, providing guidelines and recommendations useful to police, lawyers, judges, legislators, and the public. </t>
     </r>
@@ -800,7 +800,7 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>The Scientific Review Paper (SRP) Committee also supports the AP-LS core values of: continual pursuit of excellence; knowledge and application based on methods of science; outstanding service to its members and to society; social justice, diversity and inclusion; and ethical action in all that we do. Learn more about the SRC process at this link: https://h7.cl/1gFs2</t>
+      <t>The Scientific Review Paper (SRP) Committee also supports the AP-LS core values of: continual pursuit of excellence; knowledge and application based on methods of science; outstanding service to its members and to society; social justice, diversity and inclusion; and ethical action in all that we do. [Click here to view full SRP terms of reference](https://drive.google.com/file/d/1929eekRdYy7eciX-X72Oit05ZNefTLm4/view?usp=sharing)</t>
     </r>
   </si>
 </sst>
@@ -808,7 +808,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -974,6 +974,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -1316,7 +1322,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1328,6 +1334,7 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1706,7 +1713,9 @@
   <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="100.5" customWidth="1"/>
+    <col min="4" max="4" width="124.6640625" customWidth="1"/>
+    <col min="8" max="8" width="10.1640625" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
@@ -1816,7 +1825,7 @@
         <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="E4" t="s">
         <v>33</v>
@@ -1845,7 +1854,7 @@
         <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D5" t="s">
         <v>41</v>
@@ -1941,10 +1950,10 @@
         <v>69</v>
       </c>
       <c r="D8" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E8" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="F8" t="s">
         <v>70</v>
@@ -2008,7 +2017,7 @@
         <v>87</v>
       </c>
       <c r="E10" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F10" t="s">
         <v>88</v>
@@ -2087,7 +2096,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>112</v>
       </c>
@@ -2182,10 +2191,10 @@
         <v>139</v>
       </c>
       <c r="C16" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D16" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E16" t="s">
         <v>140</v>
@@ -2293,172 +2302,172 @@
         <v>169</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>170</v>
       </c>
       <c r="B20" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>233</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="G20" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="H20" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="J20" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="K20" t="s">
         <v>231</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="J20" t="s">
-        <v>171</v>
-      </c>
-      <c r="K20" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>171</v>
+      </c>
+      <c r="B21" t="s">
+        <v>172</v>
+      </c>
+      <c r="C21" t="s">
         <v>173</v>
       </c>
-      <c r="B21" t="s">
+      <c r="E21" t="s">
         <v>174</v>
       </c>
-      <c r="C21" t="s">
+      <c r="F21" t="s">
         <v>175</v>
       </c>
-      <c r="E21" t="s">
+      <c r="G21" t="s">
         <v>176</v>
       </c>
-      <c r="F21" t="s">
+      <c r="H21" t="s">
         <v>177</v>
       </c>
-      <c r="G21" t="s">
+      <c r="J21" t="s">
         <v>178</v>
       </c>
-      <c r="H21" t="s">
+      <c r="K21" t="s">
         <v>179</v>
-      </c>
-      <c r="J21" t="s">
-        <v>180</v>
-      </c>
-      <c r="K21" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>180</v>
+      </c>
+      <c r="B22" t="s">
+        <v>181</v>
+      </c>
+      <c r="C22" t="s">
         <v>182</v>
       </c>
-      <c r="B22" t="s">
+      <c r="J22" t="s">
         <v>183</v>
       </c>
-      <c r="C22" t="s">
+      <c r="K22" t="s">
         <v>184</v>
-      </c>
-      <c r="J22" t="s">
-        <v>185</v>
-      </c>
-      <c r="K22" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>185</v>
+      </c>
+      <c r="B23" t="s">
+        <v>186</v>
+      </c>
+      <c r="C23" t="s">
         <v>187</v>
       </c>
-      <c r="B23" t="s">
+      <c r="D23" t="s">
         <v>188</v>
       </c>
-      <c r="C23" t="s">
+      <c r="E23" t="s">
         <v>189</v>
       </c>
-      <c r="D23" t="s">
+      <c r="F23" t="s">
         <v>190</v>
       </c>
-      <c r="E23" t="s">
+      <c r="G23" t="s">
         <v>191</v>
-      </c>
-      <c r="F23" t="s">
-        <v>192</v>
-      </c>
-      <c r="G23" t="s">
-        <v>193</v>
       </c>
       <c r="H23" t="s">
         <v>55</v>
       </c>
       <c r="J23" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="K23" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
+        <v>194</v>
+      </c>
+      <c r="B24" t="s">
+        <v>195</v>
+      </c>
+      <c r="C24" t="s">
         <v>196</v>
       </c>
-      <c r="B24" t="s">
+      <c r="D24" t="s">
         <v>197</v>
       </c>
-      <c r="C24" t="s">
+      <c r="E24" t="s">
         <v>198</v>
-      </c>
-      <c r="D24" t="s">
-        <v>199</v>
-      </c>
-      <c r="E24" t="s">
-        <v>200</v>
       </c>
       <c r="F24" t="s">
         <v>116</v>
       </c>
       <c r="G24" t="s">
+        <v>199</v>
+      </c>
+      <c r="H24" t="s">
+        <v>200</v>
+      </c>
+      <c r="J24" t="s">
         <v>201</v>
       </c>
-      <c r="H24" t="s">
+      <c r="K24" t="s">
         <v>202</v>
-      </c>
-      <c r="J24" t="s">
-        <v>203</v>
-      </c>
-      <c r="K24" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>203</v>
+      </c>
+      <c r="B25" t="s">
+        <v>204</v>
+      </c>
+      <c r="C25" t="s">
         <v>205</v>
       </c>
-      <c r="B25" t="s">
+      <c r="D25" t="s">
         <v>206</v>
       </c>
-      <c r="C25" t="s">
+      <c r="E25" t="s">
         <v>207</v>
       </c>
-      <c r="D25" t="s">
+      <c r="F25" t="s">
         <v>208</v>
       </c>
-      <c r="E25" t="s">
+      <c r="G25" t="s">
         <v>209</v>
       </c>
-      <c r="F25" t="s">
+      <c r="H25" t="s">
         <v>210</v>
-      </c>
-      <c r="G25" t="s">
-        <v>211</v>
-      </c>
-      <c r="H25" t="s">
-        <v>212</v>
       </c>
       <c r="J25" t="s">
         <v>168</v>
@@ -2469,25 +2478,25 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
+        <v>211</v>
+      </c>
+      <c r="B26" t="s">
+        <v>212</v>
+      </c>
+      <c r="C26" t="s">
         <v>213</v>
       </c>
-      <c r="B26" t="s">
+      <c r="E26" t="s">
         <v>214</v>
       </c>
-      <c r="C26" t="s">
+      <c r="F26" t="s">
         <v>215</v>
       </c>
-      <c r="E26" t="s">
+      <c r="G26" t="s">
         <v>216</v>
       </c>
-      <c r="F26" t="s">
+      <c r="H26" t="s">
         <v>217</v>
-      </c>
-      <c r="G26" t="s">
-        <v>218</v>
-      </c>
-      <c r="H26" t="s">
-        <v>219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>